<commit_message>
#417 add type label in solution component export
</commit_message>
<xml_diff>
--- a/SolutionItems/Customisations.xlsx
+++ b/SolutionItems/Customisations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joseph.mcgregor-macd\source\repos\XRM-Developer-Tool\SolutionItems\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JosephMcGregor-Macdo\source\repos\josephmcmac\JM-Dataverse-Toolbelt\SolutionItems\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6214ED1B-4E0E-4520-B882-1AD9E45BEFA4}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D72EC457-F0F4-436A-9591-78CD104E2B50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="64680" yWindow="-3465" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Record Types" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="98">
   <si>
     <t>Relationship Name</t>
   </si>
@@ -308,13 +308,22 @@
   </si>
   <si>
     <t>Ignore</t>
+  </si>
+  <si>
+    <t>Test Entity One</t>
+  </si>
+  <si>
+    <t>Integer Format</t>
+  </si>
+  <si>
+    <t>Duration</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -329,6 +338,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -354,7 +369,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -373,9 +388,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -413,9 +428,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -448,26 +463,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -500,26 +498,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -694,16 +675,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="17.88671875" customWidth="1"/>
-    <col min="3" max="3" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.90625" customWidth="1"/>
+    <col min="3" max="3" width="23.36328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23" customWidth="1"/>
-    <col min="6" max="6" width="8.109375" customWidth="1"/>
+    <col min="6" max="6" width="8.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>94</v>
       </c>
@@ -741,7 +722,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="b">
         <v>0</v>
       </c>
@@ -779,7 +760,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" t="b">
         <v>0</v>
       </c>
@@ -817,7 +798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" t="b">
         <v>0</v>
       </c>
@@ -863,27 +844,29 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:U20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:V27"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="25.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.5546875" customWidth="1"/>
+    <col min="2" max="2" width="25.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.54296875" customWidth="1"/>
     <col min="4" max="4" width="21" customWidth="1"/>
-    <col min="5" max="5" width="15.5546875" customWidth="1"/>
-    <col min="6" max="6" width="41.33203125" customWidth="1"/>
+    <col min="5" max="5" width="15.54296875" customWidth="1"/>
+    <col min="6" max="6" width="41.36328125" customWidth="1"/>
     <col min="7" max="7" width="24" customWidth="1"/>
-    <col min="8" max="8" width="13.109375" customWidth="1"/>
-    <col min="9" max="9" width="8.109375" customWidth="1"/>
-    <col min="10" max="12" width="12.33203125" customWidth="1"/>
-    <col min="13" max="14" width="15.6640625" customWidth="1"/>
-    <col min="15" max="15" width="14.5546875" customWidth="1"/>
-    <col min="16" max="17" width="12.33203125" customWidth="1"/>
-    <col min="18" max="18" width="13.33203125" customWidth="1"/>
-    <col min="19" max="20" width="13.109375" customWidth="1"/>
-    <col min="21" max="21" width="45" customWidth="1"/>
+    <col min="8" max="8" width="13.08984375" customWidth="1"/>
+    <col min="9" max="9" width="8.08984375" customWidth="1"/>
+    <col min="10" max="12" width="12.36328125" customWidth="1"/>
+    <col min="13" max="14" width="15.6328125" customWidth="1"/>
+    <col min="15" max="15" width="14.54296875" customWidth="1"/>
+    <col min="16" max="16" width="12.36328125" customWidth="1"/>
+    <col min="17" max="17" width="10.7265625" customWidth="1"/>
+    <col min="18" max="18" width="12.36328125" customWidth="1"/>
+    <col min="19" max="19" width="13.36328125" customWidth="1"/>
+    <col min="20" max="21" width="13.08984375" customWidth="1"/>
+    <col min="22" max="22" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>94</v>
       </c>
@@ -932,25 +915,28 @@
       <c r="P1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="R1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>48</v>
@@ -997,9 +983,7 @@
       <c r="P2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q2" s="1">
-        <v>0</v>
-      </c>
+      <c r="Q2" s="2"/>
       <c r="R2" s="1">
         <v>0</v>
       </c>
@@ -1009,13 +993,16 @@
       <c r="T2" s="1">
         <v>0</v>
       </c>
-      <c r="U2" s="1" t="s">
+      <c r="U2" s="1">
+        <v>0</v>
+      </c>
+      <c r="V2" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
         <v>48</v>
@@ -1062,9 +1049,6 @@
       <c r="P3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q3" s="1">
-        <v>0</v>
-      </c>
       <c r="R3" s="1">
         <v>0</v>
       </c>
@@ -1074,13 +1058,16 @@
       <c r="T3" s="1">
         <v>0</v>
       </c>
-      <c r="U3" s="1" t="s">
+      <c r="U3" s="1">
+        <v>0</v>
+      </c>
+      <c r="V3" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B4" t="s">
         <v>48</v>
@@ -1127,25 +1114,25 @@
       <c r="P4" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q4" s="1">
-        <v>0</v>
-      </c>
       <c r="R4" s="1">
+        <v>0</v>
+      </c>
+      <c r="S4" s="1">
         <v>-100000000</v>
       </c>
-      <c r="S4" s="1">
+      <c r="T4" s="1">
         <v>100000000</v>
       </c>
-      <c r="T4" s="1">
-        <v>0</v>
-      </c>
-      <c r="U4" s="1" t="s">
+      <c r="U4" s="1">
+        <v>0</v>
+      </c>
+      <c r="V4" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B5" t="s">
         <v>48</v>
@@ -1192,25 +1179,25 @@
       <c r="P5" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q5" s="1">
-        <v>0</v>
-      </c>
       <c r="R5" s="1">
+        <v>0</v>
+      </c>
+      <c r="S5" s="1">
         <v>-100000000</v>
       </c>
-      <c r="S5" s="1">
+      <c r="T5" s="1">
         <v>100000000</v>
       </c>
-      <c r="T5" s="1">
-        <v>0</v>
-      </c>
-      <c r="U5" s="1" t="s">
+      <c r="U5" s="1">
+        <v>0</v>
+      </c>
+      <c r="V5" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B6" t="s">
         <v>48</v>
@@ -1257,25 +1244,25 @@
       <c r="P6" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q6" s="1">
-        <v>0</v>
-      </c>
       <c r="R6" s="1">
+        <v>0</v>
+      </c>
+      <c r="S6" s="1">
         <v>-100000000</v>
       </c>
-      <c r="S6" s="1">
+      <c r="T6" s="1">
         <v>100000000</v>
       </c>
-      <c r="T6" s="1">
-        <v>0</v>
-      </c>
-      <c r="U6" s="1" t="s">
+      <c r="U6" s="1">
+        <v>0</v>
+      </c>
+      <c r="V6" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B7" t="s">
         <v>48</v>
@@ -1322,25 +1309,25 @@
       <c r="P7" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q7" s="1">
-        <v>0</v>
-      </c>
       <c r="R7" s="1">
+        <v>0</v>
+      </c>
+      <c r="S7" s="1">
         <v>-100000000</v>
       </c>
-      <c r="S7" s="1">
+      <c r="T7" s="1">
         <v>100000000</v>
       </c>
-      <c r="T7" s="1">
-        <v>0</v>
-      </c>
-      <c r="U7" s="1" t="s">
+      <c r="U7" s="1">
+        <v>0</v>
+      </c>
+      <c r="V7" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
         <v>48</v>
@@ -1387,25 +1374,25 @@
       <c r="P8" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q8" s="1">
-        <v>0</v>
-      </c>
       <c r="R8" s="1">
+        <v>0</v>
+      </c>
+      <c r="S8" s="1">
         <v>-100000000</v>
       </c>
-      <c r="S8" s="1">
+      <c r="T8" s="1">
         <v>100000000</v>
       </c>
-      <c r="T8" s="1">
-        <v>0</v>
-      </c>
-      <c r="U8" s="1" t="s">
+      <c r="U8" s="1">
+        <v>0</v>
+      </c>
+      <c r="V8" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B9" t="s">
         <v>48</v>
@@ -1452,25 +1439,25 @@
       <c r="P9" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q9" s="1">
-        <v>0</v>
-      </c>
       <c r="R9" s="1">
+        <v>0</v>
+      </c>
+      <c r="S9" s="1">
         <v>-100000000</v>
       </c>
-      <c r="S9" s="1">
+      <c r="T9" s="1">
         <v>100000000</v>
       </c>
-      <c r="T9" s="1">
-        <v>0</v>
-      </c>
-      <c r="U9" s="1" t="s">
+      <c r="U9" s="1">
+        <v>0</v>
+      </c>
+      <c r="V9" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B10" t="s">
         <v>48</v>
@@ -1517,25 +1504,25 @@
       <c r="P10" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q10" s="1">
-        <v>0</v>
-      </c>
       <c r="R10" s="1">
+        <v>0</v>
+      </c>
+      <c r="S10" s="1">
         <v>-100000000</v>
       </c>
-      <c r="S10" s="1">
+      <c r="T10" s="1">
         <v>100000000</v>
       </c>
-      <c r="T10" s="1">
-        <v>0</v>
-      </c>
-      <c r="U10" s="1" t="s">
+      <c r="U10" s="1">
+        <v>0</v>
+      </c>
+      <c r="V10" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B11" t="s">
         <v>48</v>
@@ -1582,25 +1569,25 @@
       <c r="P11" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q11" s="1">
-        <v>0</v>
-      </c>
       <c r="R11" s="1">
+        <v>0</v>
+      </c>
+      <c r="S11" s="1">
         <v>-100000000</v>
       </c>
-      <c r="S11" s="1">
+      <c r="T11" s="1">
         <v>100000000</v>
       </c>
-      <c r="T11" s="1">
-        <v>0</v>
-      </c>
-      <c r="U11" s="1" t="s">
+      <c r="U11" s="1">
+        <v>0</v>
+      </c>
+      <c r="V11" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B12" t="s">
         <v>48</v>
@@ -1647,25 +1634,25 @@
       <c r="P12" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q12" s="1">
-        <v>1</v>
-      </c>
       <c r="R12" s="1">
+        <v>1</v>
+      </c>
+      <c r="S12" s="1">
         <v>-100000000</v>
       </c>
-      <c r="S12" s="1">
+      <c r="T12" s="1">
         <v>100000000</v>
       </c>
-      <c r="T12" s="1">
-        <v>0</v>
-      </c>
-      <c r="U12" s="1" t="s">
+      <c r="U12" s="1">
+        <v>0</v>
+      </c>
+      <c r="V12" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B13" t="s">
         <v>48</v>
@@ -1712,25 +1699,25 @@
       <c r="P13" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q13" s="1">
-        <v>0</v>
-      </c>
       <c r="R13" s="1">
+        <v>0</v>
+      </c>
+      <c r="S13" s="1">
         <v>-100000000</v>
       </c>
-      <c r="S13" s="1">
+      <c r="T13" s="1">
         <v>100000000</v>
       </c>
-      <c r="T13" s="1">
-        <v>0</v>
-      </c>
-      <c r="U13" s="1" t="s">
+      <c r="U13" s="1">
+        <v>0</v>
+      </c>
+      <c r="V13" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B14" t="s">
         <v>48</v>
@@ -1777,25 +1764,25 @@
       <c r="P14" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q14" s="1">
-        <v>0</v>
-      </c>
       <c r="R14" s="1">
+        <v>0</v>
+      </c>
+      <c r="S14" s="1">
         <v>-100000000</v>
       </c>
-      <c r="S14" s="1">
+      <c r="T14" s="1">
         <v>100000000</v>
       </c>
-      <c r="T14" s="1">
-        <v>0</v>
-      </c>
-      <c r="U14" s="1" t="s">
+      <c r="U14" s="1">
+        <v>0</v>
+      </c>
+      <c r="V14" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B15" t="s">
         <v>48</v>
@@ -1842,25 +1829,25 @@
       <c r="P15" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q15" s="1">
-        <v>0</v>
-      </c>
       <c r="R15" s="1">
+        <v>0</v>
+      </c>
+      <c r="S15" s="1">
         <v>-100000000</v>
       </c>
-      <c r="S15" s="1">
+      <c r="T15" s="1">
         <v>100000000</v>
       </c>
-      <c r="T15" s="1">
-        <v>0</v>
-      </c>
-      <c r="U15" s="1" t="s">
+      <c r="U15" s="1">
+        <v>0</v>
+      </c>
+      <c r="V15" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B16" t="s">
         <v>48</v>
@@ -1907,9 +1894,6 @@
       <c r="P16" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q16" s="1">
-        <v>0</v>
-      </c>
       <c r="R16" s="1">
         <v>0</v>
       </c>
@@ -1919,13 +1903,16 @@
       <c r="T16" s="1">
         <v>0</v>
       </c>
-      <c r="U16" s="1" t="s">
+      <c r="U16" s="1">
+        <v>0</v>
+      </c>
+      <c r="V16" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B17" t="s">
         <v>80</v>
@@ -1972,9 +1959,7 @@
       <c r="P17" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q17" s="1">
-        <v>0</v>
-      </c>
+      <c r="Q17"/>
       <c r="R17" s="1">
         <v>0</v>
       </c>
@@ -1984,13 +1969,16 @@
       <c r="T17" s="1">
         <v>0</v>
       </c>
-      <c r="U17" s="1" t="s">
+      <c r="U17" s="1">
+        <v>0</v>
+      </c>
+      <c r="V17" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B18" t="s">
         <v>80</v>
@@ -2037,9 +2025,7 @@
       <c r="P18" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q18" s="1">
-        <v>0</v>
-      </c>
+      <c r="Q18"/>
       <c r="R18" s="1">
         <v>0</v>
       </c>
@@ -2049,11 +2035,14 @@
       <c r="T18" s="1">
         <v>0</v>
       </c>
-      <c r="U18" s="1" t="s">
+      <c r="U18" s="1">
+        <v>0</v>
+      </c>
+      <c r="V18" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="b">
         <v>0</v>
       </c>
@@ -2102,9 +2091,7 @@
       <c r="P19" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q19" s="1">
-        <v>0</v>
-      </c>
+      <c r="Q19"/>
       <c r="R19" s="1">
         <v>0</v>
       </c>
@@ -2114,11 +2101,14 @@
       <c r="T19" s="1">
         <v>0</v>
       </c>
-      <c r="U19" s="1" t="s">
+      <c r="U19" s="1">
+        <v>0</v>
+      </c>
+      <c r="V19" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="20" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="b">
         <v>0</v>
       </c>
@@ -2146,12 +2136,8 @@
       <c r="I20" t="b">
         <v>0</v>
       </c>
-      <c r="J20" t="b">
-        <v>1</v>
-      </c>
-      <c r="K20">
-        <v>1</v>
-      </c>
+      <c r="J20"/>
+      <c r="K20"/>
       <c r="L20">
         <v>200</v>
       </c>
@@ -2167,8 +2153,8 @@
       <c r="P20" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Q20" s="1">
-        <v>0</v>
+      <c r="Q20" t="s">
+        <v>97</v>
       </c>
       <c r="R20" s="1">
         <v>0</v>
@@ -2179,17 +2165,401 @@
       <c r="T20" s="1">
         <v>0</v>
       </c>
-      <c r="U20" s="1" t="s">
+      <c r="U20" s="1">
+        <v>0</v>
+      </c>
+      <c r="V20" s="1" t="s">
         <v>29</v>
       </c>
     </row>
+    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="B21" t="s">
+        <v>81</v>
+      </c>
+      <c r="C21" t="s">
+        <v>57</v>
+      </c>
+      <c r="D21" t="s">
+        <v>95</v>
+      </c>
+      <c r="E21" t="s">
+        <v>59</v>
+      </c>
+      <c r="F21" t="s">
+        <v>55</v>
+      </c>
+      <c r="G21" t="b">
+        <v>0</v>
+      </c>
+      <c r="H21" t="b">
+        <v>0</v>
+      </c>
+      <c r="I21" t="b">
+        <v>0</v>
+      </c>
+      <c r="J21" t="b">
+        <v>1</v>
+      </c>
+      <c r="K21">
+        <v>1</v>
+      </c>
+      <c r="L21">
+        <v>200</v>
+      </c>
+      <c r="M21" t="s">
+        <v>48</v>
+      </c>
+      <c r="N21" t="b">
+        <v>1</v>
+      </c>
+      <c r="O21">
+        <v>202</v>
+      </c>
+      <c r="P21" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="R21" s="1">
+        <v>0</v>
+      </c>
+      <c r="S21" s="1">
+        <v>-100000000</v>
+      </c>
+      <c r="T21" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="U21" s="1">
+        <v>0</v>
+      </c>
+      <c r="V21" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="B22" t="s">
+        <v>81</v>
+      </c>
+      <c r="C22" t="s">
+        <v>71</v>
+      </c>
+      <c r="D22" t="s">
+        <v>60</v>
+      </c>
+      <c r="E22" t="s">
+        <v>60</v>
+      </c>
+      <c r="F22" t="s">
+        <v>55</v>
+      </c>
+      <c r="G22" t="b">
+        <v>0</v>
+      </c>
+      <c r="H22" t="b">
+        <v>0</v>
+      </c>
+      <c r="I22" t="b">
+        <v>0</v>
+      </c>
+      <c r="J22" t="b">
+        <v>1</v>
+      </c>
+      <c r="M22" t="s">
+        <v>56</v>
+      </c>
+      <c r="N22" t="b">
+        <v>1</v>
+      </c>
+      <c r="O22">
+        <v>203</v>
+      </c>
+      <c r="P22" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="R22" s="1">
+        <v>0</v>
+      </c>
+      <c r="S22" s="1">
+        <v>-100000000</v>
+      </c>
+      <c r="T22" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="U22" s="1">
+        <v>0</v>
+      </c>
+      <c r="V22" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="B23" t="s">
+        <v>81</v>
+      </c>
+      <c r="C23" t="s">
+        <v>72</v>
+      </c>
+      <c r="D23" t="s">
+        <v>61</v>
+      </c>
+      <c r="E23" t="s">
+        <v>61</v>
+      </c>
+      <c r="F23" t="s">
+        <v>55</v>
+      </c>
+      <c r="G23" t="b">
+        <v>0</v>
+      </c>
+      <c r="H23" t="b">
+        <v>0</v>
+      </c>
+      <c r="I23" t="b">
+        <v>0</v>
+      </c>
+      <c r="J23" t="b">
+        <v>1</v>
+      </c>
+      <c r="M23" t="s">
+        <v>56</v>
+      </c>
+      <c r="N23" t="b">
+        <v>1</v>
+      </c>
+      <c r="O23">
+        <v>204</v>
+      </c>
+      <c r="P23" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="R23" s="1">
+        <v>0</v>
+      </c>
+      <c r="S23" s="1">
+        <v>-100000000</v>
+      </c>
+      <c r="T23" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="U23" s="1">
+        <v>0</v>
+      </c>
+      <c r="V23" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="B24" t="s">
+        <v>81</v>
+      </c>
+      <c r="C24" t="s">
+        <v>73</v>
+      </c>
+      <c r="D24" t="s">
+        <v>66</v>
+      </c>
+      <c r="E24" t="s">
+        <v>66</v>
+      </c>
+      <c r="F24" t="s">
+        <v>55</v>
+      </c>
+      <c r="G24" t="b">
+        <v>0</v>
+      </c>
+      <c r="H24" t="b">
+        <v>0</v>
+      </c>
+      <c r="I24" t="b">
+        <v>0</v>
+      </c>
+      <c r="J24" t="b">
+        <v>1</v>
+      </c>
+      <c r="M24" t="s">
+        <v>56</v>
+      </c>
+      <c r="N24" t="b">
+        <v>1</v>
+      </c>
+      <c r="O24">
+        <v>205</v>
+      </c>
+      <c r="P24" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="R24" s="1">
+        <v>0</v>
+      </c>
+      <c r="S24" s="1">
+        <v>-100000000</v>
+      </c>
+      <c r="T24" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="U24" s="1">
+        <v>0</v>
+      </c>
+      <c r="V24" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="B25" t="s">
+        <v>81</v>
+      </c>
+      <c r="C25" t="s">
+        <v>74</v>
+      </c>
+      <c r="D25" t="s">
+        <v>67</v>
+      </c>
+      <c r="E25" t="s">
+        <v>67</v>
+      </c>
+      <c r="F25" t="s">
+        <v>55</v>
+      </c>
+      <c r="G25" t="b">
+        <v>0</v>
+      </c>
+      <c r="H25" t="b">
+        <v>0</v>
+      </c>
+      <c r="I25" t="b">
+        <v>0</v>
+      </c>
+      <c r="J25" t="b">
+        <v>1</v>
+      </c>
+      <c r="K25">
+        <v>1</v>
+      </c>
+      <c r="L25">
+        <v>200</v>
+      </c>
+      <c r="M25" t="s">
+        <v>56</v>
+      </c>
+      <c r="N25" t="b">
+        <v>1</v>
+      </c>
+      <c r="O25">
+        <v>206</v>
+      </c>
+      <c r="P25" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="R25" s="1">
+        <v>0</v>
+      </c>
+      <c r="S25" s="1">
+        <v>-100000000</v>
+      </c>
+      <c r="T25" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="U25" s="1">
+        <v>0</v>
+      </c>
+      <c r="V25" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="B26" t="s">
+        <v>81</v>
+      </c>
+      <c r="C26" t="s">
+        <v>75</v>
+      </c>
+      <c r="D26" t="s">
+        <v>68</v>
+      </c>
+      <c r="E26" t="s">
+        <v>68</v>
+      </c>
+      <c r="F26" t="s">
+        <v>55</v>
+      </c>
+      <c r="G26" t="b">
+        <v>0</v>
+      </c>
+      <c r="H26" t="b">
+        <v>0</v>
+      </c>
+      <c r="I26" t="b">
+        <v>0</v>
+      </c>
+      <c r="J26" t="b">
+        <v>1</v>
+      </c>
+      <c r="K26">
+        <v>1</v>
+      </c>
+      <c r="L26">
+        <v>200</v>
+      </c>
+      <c r="M26" t="s">
+        <v>56</v>
+      </c>
+      <c r="N26" t="b">
+        <v>1</v>
+      </c>
+      <c r="O26">
+        <v>207</v>
+      </c>
+      <c r="P26" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>97</v>
+      </c>
+      <c r="R26" s="1">
+        <v>0</v>
+      </c>
+      <c r="S26" s="1">
+        <v>-100000000</v>
+      </c>
+      <c r="T26" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="U26" s="1">
+        <v>0</v>
+      </c>
+      <c r="V26" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="Q27" s="2"/>
+    </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E7 E16:E20 E21:E65486" xr:uid="{00000000-0002-0000-0100-000000000000}">
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E7 E16:E23 E27:E65486" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Boolean,Date,Decimal,Double,Integer,Lookup,Money,Picklist,String,Memo,Status"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P2:P20 P21:P65486" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P2:P65486" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Text,TextArea,Email,Url,TickerSymbol,Phone"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt=" - " sqref="Q2:Q1001" xr:uid="{AB5B3CC1-096D-407C-A2EC-D7113479F56E}">
+      <formula1>"None,Duration,Language,TimeZone"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2200,16 +2570,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.109375" customWidth="1"/>
+    <col min="1" max="1" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.08984375" customWidth="1"/>
     <col min="5" max="5" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -2226,54 +2596,54 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>62</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>62</v>
       </c>
-      <c r="C2" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D2" s="2">
-        <v>1</v>
-      </c>
-      <c r="E2" s="2" t="s">
+      <c r="C2" t="b">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>62</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" t="s">
         <v>62</v>
       </c>
-      <c r="C3" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D3" s="2">
+      <c r="C3" t="b">
+        <v>0</v>
+      </c>
+      <c r="D3">
         <v>2</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>62</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" t="s">
         <v>62</v>
       </c>
-      <c r="C4" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D4" s="2">
+      <c r="C4" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4">
         <v>3</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" t="s">
         <v>65</v>
       </c>
     </row>
@@ -2286,18 +2656,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="48.109375" customWidth="1"/>
-    <col min="2" max="2" width="29.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.33203125" customWidth="1"/>
-    <col min="5" max="5" width="29.109375" customWidth="1"/>
-    <col min="6" max="6" width="18.33203125" customWidth="1"/>
-    <col min="7" max="7" width="19.6640625" customWidth="1"/>
+    <col min="1" max="1" width="48.08984375" customWidth="1"/>
+    <col min="2" max="2" width="29.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.36328125" customWidth="1"/>
+    <col min="5" max="5" width="29.08984375" customWidth="1"/>
+    <col min="6" max="6" width="18.36328125" customWidth="1"/>
+    <col min="7" max="7" width="19.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2332,7 +2702,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>78</v>
       </c>
@@ -2361,7 +2731,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>79</v>
       </c>

</xml_diff>